<commit_message>
create script to migrate product stocks, fix serializer to update warehouses and fix xlsx file of warehouses script
</commit_message>
<xml_diff>
--- a/backend/sale/import_files/warehouse.xlsx
+++ b/backend/sale/import_files/warehouse.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="14">
   <si>
     <t>ID</t>
   </si>
@@ -23,9 +23,6 @@
   </si>
   <si>
     <t>ID_AGENCIA</t>
-  </si>
-  <si>
-    <t>AGENCIA</t>
   </si>
   <si>
     <t>CHAYANTA BUSTILLOS</t>
@@ -315,7 +312,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="2" width="22.75"/>
-    <col customWidth="1" min="3" max="3" width="17.13"/>
+    <col customWidth="1" min="3" max="3" width="28.5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -331,19 +328,16 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
         <v>1.0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1">
         <v>1.0</v>
@@ -360,7 +354,7 @@
         <v>5</v>
       </c>
       <c r="D3" s="1">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
@@ -370,8 +364,8 @@
       <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>6</v>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="D4" s="1">
         <v>1.0</v>
@@ -382,13 +376,13 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="D5" s="1">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="6">
@@ -396,10 +390,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D6" s="1">
         <v>1.0</v>
@@ -410,13 +404,13 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D7" s="1">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="8">
@@ -424,13 +418,13 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>10</v>
+        <v>4</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="D8" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="9">
@@ -438,10 +432,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="D9" s="1">
         <v>2.0</v>
@@ -452,13 +446,13 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D10" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="11">
@@ -466,10 +460,10 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D11" s="1">
         <v>2.0</v>
@@ -480,13 +474,13 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D12" s="1">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="13">
@@ -494,10 +488,10 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="D13" s="1">
         <v>2.0</v>

</xml_diff>